<commit_message>
docs: add manufacturing connection guide, supporting component assets, and update project documentation
</commit_message>
<xml_diff>
--- a/Gökkalkan Malzeme Listesi.xlsx
+++ b/Gökkalkan Malzeme Listesi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alperkartkaya/Documents/gokkalkan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36F707CA-CF98-0F49-8455-87C7E19D8981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B154C96-4954-F543-BC6C-453F90D9176F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2660" windowWidth="27640" windowHeight="16940" xr2:uid="{D38DFFE9-3F07-A344-9A9A-115AA25B4AE0}"/>
+    <workbookView xWindow="4360" yWindow="2660" windowWidth="27640" windowHeight="16940" xr2:uid="{D38DFFE9-3F07-A344-9A9A-115AA25B4AE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="140">
   <si>
     <t>Malzeme Numarası</t>
   </si>
@@ -369,13 +369,100 @@
   </si>
   <si>
     <t>1m</t>
+  </si>
+  <si>
+    <t>Silikon Kablo</t>
+  </si>
+  <si>
+    <t>Blendajlı Sinyal Kablosu</t>
+  </si>
+  <si>
+    <t>Kablo Taşıyıcı</t>
+  </si>
+  <si>
+    <t>Kapsül Slip Ring</t>
+  </si>
+  <si>
+    <t>Mandallı Klemens</t>
+  </si>
+  <si>
+    <t>Konnektör Seti</t>
+  </si>
+  <si>
+    <t>İzoleli Kablo Yüksük Seti</t>
+  </si>
+  <si>
+    <t>Isıyla Daralan Makaron Seti</t>
+  </si>
+  <si>
+    <t>Breadboard</t>
+  </si>
+  <si>
+    <t>Jumper Kablo Seti</t>
+  </si>
+  <si>
+    <t>Step Motor Pulse Jeneratörü</t>
+  </si>
+  <si>
+    <t>Plastik Kablo Bağı Paketi</t>
+  </si>
+  <si>
+    <t>Raspberry Pi Kamera Flex Kablosu</t>
+  </si>
+  <si>
+    <t>TTR Kablo</t>
+  </si>
+  <si>
+    <t>14 AWG, Kırmızı, 3m</t>
+  </si>
+  <si>
+    <t>14 AWG, Siyah, 3m</t>
+  </si>
+  <si>
+    <t>4x0.22, 10m</t>
+  </si>
+  <si>
+    <t>15x30mm, 1m</t>
+  </si>
+  <si>
+    <t>12 veya 24 Kanal</t>
+  </si>
+  <si>
+    <t>WAGO 221-415</t>
+  </si>
+  <si>
+    <t>XT60</t>
+  </si>
+  <si>
+    <t>Karışık Boy</t>
+  </si>
+  <si>
+    <t>830 Delikli</t>
+  </si>
+  <si>
+    <t>E-E, 40 adet</t>
+  </si>
+  <si>
+    <t>E-D, 40 adet</t>
+  </si>
+  <si>
+    <t>D-D, 40 adet</t>
+  </si>
+  <si>
+    <t>100mm/200mm</t>
+  </si>
+  <si>
+    <t>22-pin to 15-pin, 5m</t>
+  </si>
+  <si>
+    <t>2x0.75 mm²</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -410,16 +497,35 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor theme="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor theme="0" tint="-0.14999847407452621"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="19">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -649,12 +755,128 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -732,6 +954,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -963,19 +1212,19 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="medium">
           <color indexed="64"/>
         </left>
         <right style="medium">
           <color indexed="64"/>
         </right>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1021,7 +1270,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2E94E98E-4A27-0A47-ADEF-7FAFEEBBB93B}" name="Table1" displayName="Table1" ref="A1:G41" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="7" tableBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2E94E98E-4A27-0A47-ADEF-7FAFEEBBB93B}" name="Table1" displayName="Table1" ref="A1:G41" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7">
   <autoFilter ref="A1:G41" xr:uid="{2E94E98E-4A27-0A47-ADEF-7FAFEEBBB93B}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{AD75FCE8-D0DA-B646-B264-8BA62730E3D1}" name="Malzeme Numarası" dataDxfId="6"/>
@@ -1353,14 +1602,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7213261-7B14-9B47-95E3-BA38785196A4}">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.6640625" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="29.6640625" customWidth="1"/>
     <col min="4" max="4" width="33.5" customWidth="1"/>
-    <col min="5" max="5" width="23.6640625" customWidth="1"/>
+    <col min="5" max="5" width="27.1640625" customWidth="1"/>
     <col min="6" max="6" width="37.5" customWidth="1"/>
     <col min="7" max="7" width="34" customWidth="1"/>
   </cols>
@@ -1480,7 +1729,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="10">
         <v>5</v>
       </c>
@@ -1503,7 +1752,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="10">
         <v>6</v>
       </c>
@@ -1641,7 +1890,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="10">
         <v>12</v>
       </c>
@@ -1685,7 +1934,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="42" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
         <v>14</v>
       </c>
@@ -2302,6 +2551,312 @@
       </c>
       <c r="G41" s="21" t="s">
         <v>110</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B43" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="D43" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="E43" s="35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="28">
+        <v>1</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C44" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D44" s="22">
+        <v>1</v>
+      </c>
+      <c r="E44" s="34" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" s="29">
+        <v>2</v>
+      </c>
+      <c r="B45" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C45" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D45" s="22">
+        <v>1</v>
+      </c>
+      <c r="E45" s="34" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="30">
+        <v>3</v>
+      </c>
+      <c r="B46" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="C46" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D46" s="22">
+        <v>1</v>
+      </c>
+      <c r="E46" s="34" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="29">
+        <v>4</v>
+      </c>
+      <c r="B47" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="C47" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D47" s="22">
+        <v>1</v>
+      </c>
+      <c r="E47" s="34" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" s="30">
+        <v>5</v>
+      </c>
+      <c r="B48" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C48" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D48" s="22">
+        <v>1</v>
+      </c>
+      <c r="E48" s="34" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="29">
+        <v>6</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="C49" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D49" s="22">
+        <v>10</v>
+      </c>
+      <c r="E49" s="34" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="30">
+        <v>7</v>
+      </c>
+      <c r="B50" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C50" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D50" s="22">
+        <v>5</v>
+      </c>
+      <c r="E50" s="34" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="29">
+        <v>8</v>
+      </c>
+      <c r="B51" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="C51" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D51" s="22">
+        <v>1</v>
+      </c>
+      <c r="E51" s="34" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" s="30">
+        <v>9</v>
+      </c>
+      <c r="B52" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C52" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D52" s="22">
+        <v>1</v>
+      </c>
+      <c r="E52" s="34" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53" s="29">
+        <v>10</v>
+      </c>
+      <c r="B53" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C53" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D53" s="22">
+        <v>2</v>
+      </c>
+      <c r="E53" s="34" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" s="30">
+        <v>11</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C54" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D54" s="22">
+        <v>1</v>
+      </c>
+      <c r="E54" s="34" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" s="29">
+        <v>12</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C55" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D55" s="22">
+        <v>1</v>
+      </c>
+      <c r="E55" s="34" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" s="30">
+        <v>13</v>
+      </c>
+      <c r="B56" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C56" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D56" s="22">
+        <v>1</v>
+      </c>
+      <c r="E56" s="34" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" s="29">
+        <v>14</v>
+      </c>
+      <c r="B57" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C57" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D57" s="22">
+        <v>1</v>
+      </c>
+      <c r="E57" s="34" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" s="30">
+        <v>15</v>
+      </c>
+      <c r="B58" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="C58" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D58" s="22">
+        <v>2</v>
+      </c>
+      <c r="E58" s="34" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59" s="29">
+        <v>16</v>
+      </c>
+      <c r="B59" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="C59" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D59" s="22">
+        <v>1</v>
+      </c>
+      <c r="E59" s="34" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" s="29">
+        <v>17</v>
+      </c>
+      <c r="B60" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="C60" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D60" s="22">
+        <v>1</v>
+      </c>
+      <c r="E60" s="34" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2347,6 +2902,7 @@
     <hyperlink ref="F30" r:id="rId39" xr:uid="{95B51580-3CEE-454C-B564-3EF5C53E4AC6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId40"/>
   </tableParts>

</xml_diff>